<commit_message>
feat: enhance workbook generation and validation with improved header checks and instructions
</commit_message>
<xml_diff>
--- a/assets/workbook_template.xlsx
+++ b/assets/workbook_template.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="16"/>
@@ -68,7 +74,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +94,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,12 +128,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -137,7 +148,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -158,6 +169,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1378,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1451,204 +1466,1383 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>SW-OFFICE-01</t>
-        </is>
-      </c>
-      <c r="B2" s="12" t="inlineStr">
+    <row r="2" ht="52" customHeight="1">
+      <c r="A2" s="17" t="n"/>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>HOW TO USE:  Each row configures one switch port.  Set Device Name (must match the Devices sheet), choose a Port Profile, enter a Description, and fill in the VLAN column(s) required by the chosen profile.  For a 24-port switch, delete rows GigabitEthernet1/0/25 to GigabitEthernet1/0/48.  Ports NOT listed in this sheet are automatically generated as 'unused' (shutdown) ports — only add rows for ports that need explicit configuration.  The four TenGigabitEthernet uplink rows at the bottom are pre-set for port-channel uplinks; update Native VLAN, Allowed VLANs, and Port Channel No. to match your environment.</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="n"/>
+      <c r="D2" s="17" t="n"/>
+      <c r="E2" s="17" t="n"/>
+      <c r="F2" s="17" t="n"/>
+      <c r="G2" s="17" t="n"/>
+      <c r="H2" s="17" t="n"/>
+      <c r="I2" s="17" t="n"/>
+      <c r="J2" s="17" t="n"/>
+      <c r="K2" s="17" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>GigabitEthernet1/0/1</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>access-voip</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>CLIENT: PC/Phone - Desk 1</t>
-        </is>
-      </c>
-      <c r="E2" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="F2" s="12" t="n">
-        <v>30</v>
-      </c>
-      <c r="G2" s="12" t="inlineStr"/>
-      <c r="H2" s="12" t="inlineStr"/>
-      <c r="I2" s="12" t="inlineStr"/>
-      <c r="J2" s="12" t="inlineStr"/>
-      <c r="K2" s="12" t="inlineStr"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>SW-OFFICE-01</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr"/>
+      <c r="E3" s="12" t="inlineStr"/>
+      <c r="F3" s="12" t="inlineStr"/>
+      <c r="G3" s="12" t="inlineStr"/>
+      <c r="H3" s="12" t="inlineStr"/>
+      <c r="I3" s="12" t="inlineStr"/>
+      <c r="J3" s="12" t="inlineStr"/>
+      <c r="K3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>GigabitEthernet1/0/2</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>access-printer</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>PRINTER: Floor 1</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="F3" s="13" t="inlineStr"/>
-      <c r="G3" s="13" t="inlineStr"/>
-      <c r="H3" s="13" t="inlineStr"/>
-      <c r="I3" s="13" t="inlineStr"/>
-      <c r="J3" s="13" t="inlineStr"/>
-      <c r="K3" s="13" t="inlineStr"/>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>SW-OFFICE-01</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr"/>
+      <c r="E4" s="13" t="inlineStr"/>
+      <c r="F4" s="13" t="inlineStr"/>
+      <c r="G4" s="13" t="inlineStr"/>
+      <c r="H4" s="13" t="inlineStr"/>
+      <c r="I4" s="13" t="inlineStr"/>
+      <c r="J4" s="13" t="inlineStr"/>
+      <c r="K4" s="13" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>GigabitEthernet1/0/3</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>access-ap-trunk</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>WAP - Lobby</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr"/>
-      <c r="F4" s="12" t="inlineStr"/>
-      <c r="G4" s="12" t="n">
-        <v>40</v>
-      </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>10,20,40</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr"/>
+      <c r="E5" s="12" t="inlineStr"/>
+      <c r="F5" s="12" t="inlineStr"/>
+      <c r="G5" s="12" t="inlineStr"/>
+      <c r="H5" s="12" t="inlineStr"/>
+      <c r="I5" s="12" t="inlineStr"/>
+      <c r="J5" s="12" t="inlineStr"/>
+      <c r="K5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/4</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr"/>
+      <c r="E6" s="13" t="inlineStr"/>
+      <c r="F6" s="13" t="inlineStr"/>
+      <c r="G6" s="13" t="inlineStr"/>
+      <c r="H6" s="13" t="inlineStr"/>
+      <c r="I6" s="13" t="inlineStr"/>
+      <c r="J6" s="13" t="inlineStr"/>
+      <c r="K6" s="13" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/5</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr"/>
+      <c r="E7" s="12" t="inlineStr"/>
+      <c r="F7" s="12" t="inlineStr"/>
+      <c r="G7" s="12" t="inlineStr"/>
+      <c r="H7" s="12" t="inlineStr"/>
+      <c r="I7" s="12" t="inlineStr"/>
+      <c r="J7" s="12" t="inlineStr"/>
+      <c r="K7" s="12" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/6</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr"/>
+      <c r="F8" s="13" t="inlineStr"/>
+      <c r="G8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr"/>
+      <c r="J8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/7</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr"/>
+      <c r="E9" s="12" t="inlineStr"/>
+      <c r="F9" s="12" t="inlineStr"/>
+      <c r="G9" s="12" t="inlineStr"/>
+      <c r="H9" s="12" t="inlineStr"/>
+      <c r="I9" s="12" t="inlineStr"/>
+      <c r="J9" s="12" t="inlineStr"/>
+      <c r="K9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/8</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr"/>
+      <c r="J10" s="13" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/9</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr"/>
+      <c r="E11" s="12" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr"/>
+      <c r="G11" s="12" t="inlineStr"/>
+      <c r="H11" s="12" t="inlineStr"/>
+      <c r="I11" s="12" t="inlineStr"/>
+      <c r="J11" s="12" t="inlineStr"/>
+      <c r="K11" s="12" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/10</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="13" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr"/>
+      <c r="H12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr"/>
+      <c r="J12" s="13" t="inlineStr"/>
+      <c r="K12" s="13" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/11</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr"/>
+      <c r="E13" s="12" t="inlineStr"/>
+      <c r="F13" s="12" t="inlineStr"/>
+      <c r="G13" s="12" t="inlineStr"/>
+      <c r="H13" s="12" t="inlineStr"/>
+      <c r="I13" s="12" t="inlineStr"/>
+      <c r="J13" s="12" t="inlineStr"/>
+      <c r="K13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/12</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr"/>
+      <c r="E14" s="13" t="inlineStr"/>
+      <c r="F14" s="13" t="inlineStr"/>
+      <c r="G14" s="13" t="inlineStr"/>
+      <c r="H14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr"/>
+      <c r="J14" s="13" t="inlineStr"/>
+      <c r="K14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/13</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr"/>
+      <c r="E15" s="12" t="inlineStr"/>
+      <c r="F15" s="12" t="inlineStr"/>
+      <c r="G15" s="12" t="inlineStr"/>
+      <c r="H15" s="12" t="inlineStr"/>
+      <c r="I15" s="12" t="inlineStr"/>
+      <c r="J15" s="12" t="inlineStr"/>
+      <c r="K15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/14</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr"/>
+      <c r="E16" s="13" t="inlineStr"/>
+      <c r="F16" s="13" t="inlineStr"/>
+      <c r="G16" s="13" t="inlineStr"/>
+      <c r="H16" s="13" t="inlineStr"/>
+      <c r="I16" s="13" t="inlineStr"/>
+      <c r="J16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/15</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr"/>
+      <c r="E17" s="12" t="inlineStr"/>
+      <c r="F17" s="12" t="inlineStr"/>
+      <c r="G17" s="12" t="inlineStr"/>
+      <c r="H17" s="12" t="inlineStr"/>
+      <c r="I17" s="12" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr"/>
+      <c r="K17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/16</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr"/>
+      <c r="E18" s="13" t="inlineStr"/>
+      <c r="F18" s="13" t="inlineStr"/>
+      <c r="G18" s="13" t="inlineStr"/>
+      <c r="H18" s="13" t="inlineStr"/>
+      <c r="I18" s="13" t="inlineStr"/>
+      <c r="J18" s="13" t="inlineStr"/>
+      <c r="K18" s="13" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/17</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr"/>
+      <c r="E19" s="12" t="inlineStr"/>
+      <c r="F19" s="12" t="inlineStr"/>
+      <c r="G19" s="12" t="inlineStr"/>
+      <c r="H19" s="12" t="inlineStr"/>
+      <c r="I19" s="12" t="inlineStr"/>
+      <c r="J19" s="12" t="inlineStr"/>
+      <c r="K19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/18</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr"/>
+      <c r="F20" s="13" t="inlineStr"/>
+      <c r="G20" s="13" t="inlineStr"/>
+      <c r="H20" s="13" t="inlineStr"/>
+      <c r="I20" s="13" t="inlineStr"/>
+      <c r="J20" s="13" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/19</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr"/>
+      <c r="E21" s="12" t="inlineStr"/>
+      <c r="F21" s="12" t="inlineStr"/>
+      <c r="G21" s="12" t="inlineStr"/>
+      <c r="H21" s="12" t="inlineStr"/>
+      <c r="I21" s="12" t="inlineStr"/>
+      <c r="J21" s="12" t="inlineStr"/>
+      <c r="K21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/20</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr"/>
+      <c r="F22" s="13" t="inlineStr"/>
+      <c r="G22" s="13" t="inlineStr"/>
+      <c r="H22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr"/>
+      <c r="J22" s="13" t="inlineStr"/>
+      <c r="K22" s="13" t="inlineStr"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/21</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr"/>
+      <c r="E23" s="12" t="inlineStr"/>
+      <c r="F23" s="12" t="inlineStr"/>
+      <c r="G23" s="12" t="inlineStr"/>
+      <c r="H23" s="12" t="inlineStr"/>
+      <c r="I23" s="12" t="inlineStr"/>
+      <c r="J23" s="12" t="inlineStr"/>
+      <c r="K23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/22</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr"/>
+      <c r="E24" s="13" t="inlineStr"/>
+      <c r="F24" s="13" t="inlineStr"/>
+      <c r="G24" s="13" t="inlineStr"/>
+      <c r="H24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr"/>
+      <c r="J24" s="13" t="inlineStr"/>
+      <c r="K24" s="13" t="inlineStr"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/23</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr"/>
+      <c r="E25" s="12" t="inlineStr"/>
+      <c r="F25" s="12" t="inlineStr"/>
+      <c r="G25" s="12" t="inlineStr"/>
+      <c r="H25" s="12" t="inlineStr"/>
+      <c r="I25" s="12" t="inlineStr"/>
+      <c r="J25" s="12" t="inlineStr"/>
+      <c r="K25" s="12" t="inlineStr"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/24</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr"/>
+      <c r="E26" s="13" t="inlineStr"/>
+      <c r="F26" s="13" t="inlineStr"/>
+      <c r="G26" s="13" t="inlineStr"/>
+      <c r="H26" s="13" t="inlineStr"/>
+      <c r="I26" s="13" t="inlineStr"/>
+      <c r="J26" s="13" t="inlineStr"/>
+      <c r="K26" s="13" t="inlineStr"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/25</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr"/>
+      <c r="E27" s="12" t="inlineStr"/>
+      <c r="F27" s="12" t="inlineStr"/>
+      <c r="G27" s="12" t="inlineStr"/>
+      <c r="H27" s="12" t="inlineStr"/>
+      <c r="I27" s="12" t="inlineStr"/>
+      <c r="J27" s="12" t="inlineStr"/>
+      <c r="K27" s="12" t="inlineStr"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/26</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr"/>
+      <c r="E28" s="13" t="inlineStr"/>
+      <c r="F28" s="13" t="inlineStr"/>
+      <c r="G28" s="13" t="inlineStr"/>
+      <c r="H28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr"/>
+      <c r="J28" s="13" t="inlineStr"/>
+      <c r="K28" s="13" t="inlineStr"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/27</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr"/>
+      <c r="E29" s="12" t="inlineStr"/>
+      <c r="F29" s="12" t="inlineStr"/>
+      <c r="G29" s="12" t="inlineStr"/>
+      <c r="H29" s="12" t="inlineStr"/>
+      <c r="I29" s="12" t="inlineStr"/>
+      <c r="J29" s="12" t="inlineStr"/>
+      <c r="K29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/28</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr"/>
+      <c r="E30" s="13" t="inlineStr"/>
+      <c r="F30" s="13" t="inlineStr"/>
+      <c r="G30" s="13" t="inlineStr"/>
+      <c r="H30" s="13" t="inlineStr"/>
+      <c r="I30" s="13" t="inlineStr"/>
+      <c r="J30" s="13" t="inlineStr"/>
+      <c r="K30" s="13" t="inlineStr"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/29</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr"/>
+      <c r="E31" s="12" t="inlineStr"/>
+      <c r="F31" s="12" t="inlineStr"/>
+      <c r="G31" s="12" t="inlineStr"/>
+      <c r="H31" s="12" t="inlineStr"/>
+      <c r="I31" s="12" t="inlineStr"/>
+      <c r="J31" s="12" t="inlineStr"/>
+      <c r="K31" s="12" t="inlineStr"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/30</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr"/>
+      <c r="E32" s="13" t="inlineStr"/>
+      <c r="F32" s="13" t="inlineStr"/>
+      <c r="G32" s="13" t="inlineStr"/>
+      <c r="H32" s="13" t="inlineStr"/>
+      <c r="I32" s="13" t="inlineStr"/>
+      <c r="J32" s="13" t="inlineStr"/>
+      <c r="K32" s="13" t="inlineStr"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/31</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr"/>
+      <c r="E33" s="12" t="inlineStr"/>
+      <c r="F33" s="12" t="inlineStr"/>
+      <c r="G33" s="12" t="inlineStr"/>
+      <c r="H33" s="12" t="inlineStr"/>
+      <c r="I33" s="12" t="inlineStr"/>
+      <c r="J33" s="12" t="inlineStr"/>
+      <c r="K33" s="12" t="inlineStr"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/32</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr"/>
+      <c r="E34" s="13" t="inlineStr"/>
+      <c r="F34" s="13" t="inlineStr"/>
+      <c r="G34" s="13" t="inlineStr"/>
+      <c r="H34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr"/>
+      <c r="J34" s="13" t="inlineStr"/>
+      <c r="K34" s="13" t="inlineStr"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/33</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr"/>
+      <c r="E35" s="12" t="inlineStr"/>
+      <c r="F35" s="12" t="inlineStr"/>
+      <c r="G35" s="12" t="inlineStr"/>
+      <c r="H35" s="12" t="inlineStr"/>
+      <c r="I35" s="12" t="inlineStr"/>
+      <c r="J35" s="12" t="inlineStr"/>
+      <c r="K35" s="12" t="inlineStr"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/34</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr"/>
+      <c r="E36" s="13" t="inlineStr"/>
+      <c r="F36" s="13" t="inlineStr"/>
+      <c r="G36" s="13" t="inlineStr"/>
+      <c r="H36" s="13" t="inlineStr"/>
+      <c r="I36" s="13" t="inlineStr"/>
+      <c r="J36" s="13" t="inlineStr"/>
+      <c r="K36" s="13" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/35</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr"/>
+      <c r="E37" s="12" t="inlineStr"/>
+      <c r="F37" s="12" t="inlineStr"/>
+      <c r="G37" s="12" t="inlineStr"/>
+      <c r="H37" s="12" t="inlineStr"/>
+      <c r="I37" s="12" t="inlineStr"/>
+      <c r="J37" s="12" t="inlineStr"/>
+      <c r="K37" s="12" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/36</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr"/>
+      <c r="E38" s="13" t="inlineStr"/>
+      <c r="F38" s="13" t="inlineStr"/>
+      <c r="G38" s="13" t="inlineStr"/>
+      <c r="H38" s="13" t="inlineStr"/>
+      <c r="I38" s="13" t="inlineStr"/>
+      <c r="J38" s="13" t="inlineStr"/>
+      <c r="K38" s="13" t="inlineStr"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/37</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr"/>
+      <c r="E39" s="12" t="inlineStr"/>
+      <c r="F39" s="12" t="inlineStr"/>
+      <c r="G39" s="12" t="inlineStr"/>
+      <c r="H39" s="12" t="inlineStr"/>
+      <c r="I39" s="12" t="inlineStr"/>
+      <c r="J39" s="12" t="inlineStr"/>
+      <c r="K39" s="12" t="inlineStr"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/38</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr"/>
+      <c r="E40" s="13" t="inlineStr"/>
+      <c r="F40" s="13" t="inlineStr"/>
+      <c r="G40" s="13" t="inlineStr"/>
+      <c r="H40" s="13" t="inlineStr"/>
+      <c r="I40" s="13" t="inlineStr"/>
+      <c r="J40" s="13" t="inlineStr"/>
+      <c r="K40" s="13" t="inlineStr"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/39</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr"/>
+      <c r="E41" s="12" t="inlineStr"/>
+      <c r="F41" s="12" t="inlineStr"/>
+      <c r="G41" s="12" t="inlineStr"/>
+      <c r="H41" s="12" t="inlineStr"/>
+      <c r="I41" s="12" t="inlineStr"/>
+      <c r="J41" s="12" t="inlineStr"/>
+      <c r="K41" s="12" t="inlineStr"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/40</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr"/>
+      <c r="E42" s="13" t="inlineStr"/>
+      <c r="F42" s="13" t="inlineStr"/>
+      <c r="G42" s="13" t="inlineStr"/>
+      <c r="H42" s="13" t="inlineStr"/>
+      <c r="I42" s="13" t="inlineStr"/>
+      <c r="J42" s="13" t="inlineStr"/>
+      <c r="K42" s="13" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/41</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr"/>
+      <c r="E43" s="12" t="inlineStr"/>
+      <c r="F43" s="12" t="inlineStr"/>
+      <c r="G43" s="12" t="inlineStr"/>
+      <c r="H43" s="12" t="inlineStr"/>
+      <c r="I43" s="12" t="inlineStr"/>
+      <c r="J43" s="12" t="inlineStr"/>
+      <c r="K43" s="12" t="inlineStr"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/42</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr"/>
+      <c r="E44" s="13" t="inlineStr"/>
+      <c r="F44" s="13" t="inlineStr"/>
+      <c r="G44" s="13" t="inlineStr"/>
+      <c r="H44" s="13" t="inlineStr"/>
+      <c r="I44" s="13" t="inlineStr"/>
+      <c r="J44" s="13" t="inlineStr"/>
+      <c r="K44" s="13" t="inlineStr"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/43</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr"/>
+      <c r="E45" s="12" t="inlineStr"/>
+      <c r="F45" s="12" t="inlineStr"/>
+      <c r="G45" s="12" t="inlineStr"/>
+      <c r="H45" s="12" t="inlineStr"/>
+      <c r="I45" s="12" t="inlineStr"/>
+      <c r="J45" s="12" t="inlineStr"/>
+      <c r="K45" s="12" t="inlineStr"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/44</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr"/>
+      <c r="E46" s="13" t="inlineStr"/>
+      <c r="F46" s="13" t="inlineStr"/>
+      <c r="G46" s="13" t="inlineStr"/>
+      <c r="H46" s="13" t="inlineStr"/>
+      <c r="I46" s="13" t="inlineStr"/>
+      <c r="J46" s="13" t="inlineStr"/>
+      <c r="K46" s="13" t="inlineStr"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/45</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr"/>
+      <c r="E47" s="12" t="inlineStr"/>
+      <c r="F47" s="12" t="inlineStr"/>
+      <c r="G47" s="12" t="inlineStr"/>
+      <c r="H47" s="12" t="inlineStr"/>
+      <c r="I47" s="12" t="inlineStr"/>
+      <c r="J47" s="12" t="inlineStr"/>
+      <c r="K47" s="12" t="inlineStr"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/46</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr"/>
+      <c r="E48" s="13" t="inlineStr"/>
+      <c r="F48" s="13" t="inlineStr"/>
+      <c r="G48" s="13" t="inlineStr"/>
+      <c r="H48" s="13" t="inlineStr"/>
+      <c r="I48" s="13" t="inlineStr"/>
+      <c r="J48" s="13" t="inlineStr"/>
+      <c r="K48" s="13" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/47</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr"/>
+      <c r="E49" s="12" t="inlineStr"/>
+      <c r="F49" s="12" t="inlineStr"/>
+      <c r="G49" s="12" t="inlineStr"/>
+      <c r="H49" s="12" t="inlineStr"/>
+      <c r="I49" s="12" t="inlineStr"/>
+      <c r="J49" s="12" t="inlineStr"/>
+      <c r="K49" s="12" t="inlineStr"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>GigabitEthernet1/0/48</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>access-voip</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr"/>
+      <c r="E50" s="13" t="inlineStr"/>
+      <c r="F50" s="13" t="inlineStr"/>
+      <c r="G50" s="13" t="inlineStr"/>
+      <c r="H50" s="13" t="inlineStr"/>
+      <c r="I50" s="13" t="inlineStr"/>
+      <c r="J50" s="13" t="inlineStr"/>
+      <c r="K50" s="13" t="inlineStr"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>TenGigabitEthernet1/1/1</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>trunk-uplink-portchannel</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>L:Po1  R:Po1 Uplink to Core</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr"/>
+      <c r="F51" s="12" t="inlineStr"/>
+      <c r="G51" s="12" t="inlineStr"/>
+      <c r="H51" s="12" t="inlineStr"/>
+      <c r="I51" s="12" t="inlineStr">
         <is>
           <t>1.00 0.70</t>
         </is>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="J51" s="12" t="inlineStr">
         <is>
           <t>1.00 0.70</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr"/>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>SW-OFFICE-01</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>TenGigabitEthernet1/1/1</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="K51" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>TenGigabitEthernet1/1/2</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="inlineStr">
         <is>
           <t>trunk-uplink-portchannel</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D52" s="13" t="inlineStr">
         <is>
           <t>L:Po1  R:Po1 Uplink to Core</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr"/>
-      <c r="F5" s="13" t="inlineStr"/>
-      <c r="G5" s="13" t="n">
-        <v>99</v>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>10,20,40,99</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="E52" s="13" t="inlineStr"/>
+      <c r="F52" s="13" t="inlineStr"/>
+      <c r="G52" s="13" t="inlineStr"/>
+      <c r="H52" s="13" t="inlineStr"/>
+      <c r="I52" s="13" t="inlineStr">
         <is>
           <t>1.00 0.70</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J52" s="13" t="inlineStr">
         <is>
           <t>1.00 0.70</t>
         </is>
       </c>
-      <c r="K5" s="13" t="n">
+      <c r="K52" s="13" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>SW-OFFICE-01</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>TenGigabitEthernet1/1/2</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>TenGigabitEthernet1/1/3</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>trunk-uplink-portchannel</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>L:Po1  R:Po1 Uplink to Core</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr"/>
-      <c r="F6" s="12" t="inlineStr"/>
-      <c r="G6" s="12" t="n">
-        <v>99</v>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>10,20,40,99</t>
-        </is>
-      </c>
-      <c r="I6" s="12" t="inlineStr">
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>L:Po2  R:Po2 Uplink to Core</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="inlineStr"/>
+      <c r="F53" s="12" t="inlineStr"/>
+      <c r="G53" s="12" t="inlineStr"/>
+      <c r="H53" s="12" t="inlineStr"/>
+      <c r="I53" s="12" t="inlineStr">
         <is>
           <t>1.00 0.70</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr">
+      <c r="J53" s="12" t="inlineStr">
         <is>
           <t>1.00 0.70</t>
         </is>
       </c>
-      <c r="K6" s="12" t="n">
-        <v>1</v>
+      <c r="K53" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>TenGigabitEthernet1/1/4</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>trunk-uplink-portchannel</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>L:Po2  R:Po2 Uplink to Core</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr"/>
+      <c r="F54" s="13" t="inlineStr"/>
+      <c r="G54" s="13" t="inlineStr"/>
+      <c r="H54" s="13" t="inlineStr"/>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
+      <c r="K54" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:K2"/>
+  </mergeCells>
   <dataValidations count="5">
     <dataValidation sqref="A2:A300" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Value" error="Please select a valid value from the dropdown." type="list">
       <formula1>DeviceNames</formula1>

</xml_diff>

<commit_message>
feat: update versioning system and enhance workbook generation with example rows
</commit_message>
<xml_diff>
--- a/assets/workbook_template.xlsx
+++ b/assets/workbook_template.xlsx
@@ -1470,7 +1470,7 @@
       <c r="A2" s="17" t="n"/>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>HOW TO USE:  Each row configures one switch port.  Set Device Name (must match the Devices sheet), choose a Port Profile, enter a Description, and fill in the VLAN column(s) required by the chosen profile.  For a 24-port switch, delete rows GigabitEthernet1/0/25 to GigabitEthernet1/0/48.  Ports NOT listed in this sheet are automatically generated as 'unused' (shutdown) ports — only add rows for ports that need explicit configuration.  The four TenGigabitEthernet uplink rows at the bottom are pre-set for port-channel uplinks; update Native VLAN, Allowed VLANs, and Port Channel No. to match your environment.</t>
+          <t>HOW TO USE:  Each row configures one switch port.  Set Device Name (must match the Devices sheet), choose a Port Profile, enter a Description, and fill in the VLAN column(s) required by the chosen profile.  The first four rows are filled with examples showing common port types — update or replace them as needed.  For a 24-port switch, delete rows GigabitEthernet1/0/25 to GigabitEthernet1/0/48.  Ports NOT listed in this sheet are automatically generated as 'unused' (shutdown) ports — only add rows for ports that need explicit configuration.  The four TenGigabitEthernet uplink rows at the bottom are pre-set for port-channel uplinks; update Native VLAN, Allowed VLANs, and Port Channel No. to match your environment.</t>
         </is>
       </c>
       <c r="C2" s="17" t="n"/>
@@ -1499,9 +1499,17 @@
           <t>access-voip</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr"/>
-      <c r="E3" s="12" t="inlineStr"/>
-      <c r="F3" s="12" t="inlineStr"/>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>CLIENT: PC/Phone - Desk 1</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>30</v>
+      </c>
       <c r="G3" s="12" t="inlineStr"/>
       <c r="H3" s="12" t="inlineStr"/>
       <c r="I3" s="12" t="inlineStr"/>
@@ -1521,11 +1529,17 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>access-voip</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr"/>
-      <c r="E4" s="13" t="inlineStr"/>
+          <t>access-printer</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>PRINTER: Floor 1 Copier</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>20</v>
+      </c>
       <c r="F4" s="13" t="inlineStr"/>
       <c r="G4" s="13" t="inlineStr"/>
       <c r="H4" s="13" t="inlineStr"/>
@@ -1546,16 +1560,34 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>access-voip</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr"/>
+          <t>access-ap-trunk</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>WAP - Lobby</t>
+        </is>
+      </c>
       <c r="E5" s="12" t="inlineStr"/>
       <c r="F5" s="12" t="inlineStr"/>
-      <c r="G5" s="12" t="inlineStr"/>
-      <c r="H5" s="12" t="inlineStr"/>
-      <c r="I5" s="12" t="inlineStr"/>
-      <c r="J5" s="12" t="inlineStr"/>
+      <c r="G5" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>10,20,30,40</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
       <c r="K5" s="12" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -1571,11 +1603,17 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>access-voip</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr"/>
-      <c r="E6" s="13" t="inlineStr"/>
+          <t>access-user</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>CLIENT: Data only - Desk 4</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>20</v>
+      </c>
       <c r="F6" s="13" t="inlineStr"/>
       <c r="G6" s="13" t="inlineStr"/>
       <c r="H6" s="13" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: add support for port channels configuration and validation
</commit_message>
<xml_diff>
--- a/assets/workbook_template.xlsx
+++ b/assets/workbook_template.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Global Settings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="VLANs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Interfaces" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ACLs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Feature Selection" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Port-Channels" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ACLs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Feature Selection" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="VLANIDs">VLANs!$A$2:$A$300</definedName>
@@ -2905,6 +2906,141 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C55A11"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Device Name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Port Channel No.</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Native VLAN</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Allowed VLANs</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Storm Control Broadcast</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Storm Control Multicast</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Uplink to Core - Po1</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>10,20,30</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>SW-OFFICE-01</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Server Uplink - Po2</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>10,20,60</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>1.00 0.70</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="A2:A300" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Value" error="Please select a valid value from the dropdown." type="list">
+      <formula1>DeviceNames</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D300" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Value" error="Please select a valid value from the dropdown." type="list">
+      <formula1>VLANIDs</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00C00000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3121,14 +3257,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="000070C0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3309,15 +3445,32 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
+          <t>port_channels</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Logical Port-channel interfaces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
           <t>acls</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>IP access control lists — VTY and SNMP access restriction</t>
         </is>

</xml_diff>